<commit_message>
add more ОБЖ lab1
</commit_message>
<xml_diff>
--- a/ОБЖ/lab1/Определение относительной влажности воздуха аспирационным психрометром.xlsx
+++ b/ОБЖ/lab1/Определение относительной влажности воздуха аспирационным психрометром.xlsx
@@ -121,12 +121,18 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -455,695 +461,695 @@
       <c r="S1" s="2"/>
     </row>
     <row r="2" spans="1:19">
-      <c r="A2" s="1"/>
-      <c r="B2" s="1">
+      <c r="A2" s="3"/>
+      <c r="B2" s="3">
         <v>8</v>
       </c>
-      <c r="C2" s="1">
+      <c r="C2" s="3">
         <v>9</v>
       </c>
-      <c r="D2" s="1">
+      <c r="D2" s="3">
         <v>10</v>
       </c>
-      <c r="E2" s="1">
+      <c r="E2" s="3">
         <v>11</v>
       </c>
-      <c r="F2" s="1">
+      <c r="F2" s="3">
         <v>12</v>
       </c>
-      <c r="G2" s="1">
+      <c r="G2" s="3">
         <v>13</v>
       </c>
-      <c r="H2" s="1">
+      <c r="H2" s="3">
         <v>14</v>
       </c>
-      <c r="I2" s="1">
+      <c r="I2" s="3">
         <v>15</v>
       </c>
-      <c r="J2" s="1">
+      <c r="J2" s="3">
         <v>16</v>
       </c>
-      <c r="K2" s="1">
+      <c r="K2" s="3">
         <v>17</v>
       </c>
-      <c r="L2" s="1">
+      <c r="L2" s="3">
         <v>18</v>
       </c>
-      <c r="M2" s="1">
+      <c r="M2" s="3">
         <v>19</v>
       </c>
-      <c r="N2" s="1">
+      <c r="N2" s="3">
         <v>20</v>
       </c>
-      <c r="O2" s="1">
+      <c r="O2" s="3">
         <v>21</v>
       </c>
-      <c r="P2" s="1">
+      <c r="P2" s="3">
         <v>22</v>
       </c>
-      <c r="Q2" s="1">
+      <c r="Q2" s="3">
         <v>23</v>
       </c>
-      <c r="R2" s="1">
+      <c r="R2" s="3">
         <v>24</v>
       </c>
-      <c r="S2" s="1">
+      <c r="S2" s="3">
         <v>25</v>
       </c>
     </row>
     <row r="3" spans="1:19" ht="15" customHeight="1">
-      <c r="A3" s="1"/>
-      <c r="B3" s="2" t="s">
+      <c r="A3" s="3"/>
+      <c r="B3" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2"/>
-      <c r="E3" s="2"/>
-      <c r="F3" s="2"/>
-      <c r="G3" s="2"/>
-      <c r="H3" s="2"/>
-      <c r="I3" s="2"/>
-      <c r="J3" s="2"/>
-      <c r="K3" s="2"/>
-      <c r="L3" s="2"/>
-      <c r="M3" s="2"/>
-      <c r="N3" s="2"/>
-      <c r="O3" s="2"/>
-      <c r="P3" s="2"/>
-      <c r="Q3" s="2"/>
-      <c r="R3" s="2"/>
-      <c r="S3" s="2"/>
+      <c r="C3" s="4"/>
+      <c r="D3" s="4"/>
+      <c r="E3" s="4"/>
+      <c r="F3" s="4"/>
+      <c r="G3" s="4"/>
+      <c r="H3" s="4"/>
+      <c r="I3" s="4"/>
+      <c r="J3" s="4"/>
+      <c r="K3" s="4"/>
+      <c r="L3" s="4"/>
+      <c r="M3" s="4"/>
+      <c r="N3" s="4"/>
+      <c r="O3" s="4"/>
+      <c r="P3" s="4"/>
+      <c r="Q3" s="4"/>
+      <c r="R3" s="4"/>
+      <c r="S3" s="4"/>
     </row>
     <row r="4" spans="1:19">
-      <c r="A4" s="1">
+      <c r="A4" s="3">
         <v>15</v>
       </c>
-      <c r="B4" s="1">
+      <c r="B4" s="3">
         <v>36</v>
       </c>
-      <c r="C4" s="1">
+      <c r="C4" s="3">
         <v>44</v>
       </c>
-      <c r="D4" s="1">
+      <c r="D4" s="3">
         <v>52</v>
       </c>
-      <c r="E4" s="1">
+      <c r="E4" s="3">
         <v>61</v>
       </c>
-      <c r="F4" s="1">
+      <c r="F4" s="3">
         <v>71</v>
       </c>
-      <c r="G4" s="1">
+      <c r="G4" s="3">
         <v>80</v>
       </c>
-      <c r="H4" s="1">
+      <c r="H4" s="3">
         <v>90</v>
       </c>
-      <c r="I4" s="1">
+      <c r="I4" s="3">
         <v>100</v>
       </c>
-      <c r="J4" s="1"/>
-      <c r="K4" s="1"/>
-      <c r="L4" s="1"/>
-      <c r="M4" s="1"/>
-      <c r="N4" s="1"/>
-      <c r="O4" s="1"/>
-      <c r="P4" s="1"/>
-      <c r="Q4" s="1"/>
-      <c r="R4" s="1"/>
-      <c r="S4" s="1"/>
+      <c r="J4" s="3"/>
+      <c r="K4" s="3"/>
+      <c r="L4" s="3"/>
+      <c r="M4" s="3"/>
+      <c r="N4" s="3"/>
+      <c r="O4" s="3"/>
+      <c r="P4" s="3"/>
+      <c r="Q4" s="3"/>
+      <c r="R4" s="3"/>
+      <c r="S4" s="3"/>
     </row>
     <row r="5" spans="1:19">
-      <c r="A5" s="1">
+      <c r="A5" s="3">
         <v>16</v>
       </c>
-      <c r="B5" s="1">
+      <c r="B5" s="3">
         <v>30</v>
       </c>
-      <c r="C5" s="1">
+      <c r="C5" s="3">
         <v>37</v>
       </c>
-      <c r="D5" s="1">
+      <c r="D5" s="3">
         <v>46</v>
       </c>
-      <c r="E5" s="1">
+      <c r="E5" s="3">
         <v>54</v>
       </c>
-      <c r="F5" s="1">
+      <c r="F5" s="3">
         <v>63</v>
       </c>
-      <c r="G5" s="1">
+      <c r="G5" s="3">
         <v>71</v>
       </c>
-      <c r="H5" s="1">
+      <c r="H5" s="3">
         <v>81</v>
       </c>
-      <c r="I5" s="1">
+      <c r="I5" s="3">
         <v>90</v>
       </c>
-      <c r="J5" s="1">
+      <c r="J5" s="3">
         <v>100</v>
       </c>
-      <c r="K5" s="1"/>
-      <c r="L5" s="1"/>
-      <c r="M5" s="1"/>
-      <c r="N5" s="1"/>
-      <c r="O5" s="1"/>
-      <c r="P5" s="1"/>
-      <c r="Q5" s="1"/>
-      <c r="R5" s="1"/>
-      <c r="S5" s="1"/>
+      <c r="K5" s="3"/>
+      <c r="L5" s="3"/>
+      <c r="M5" s="3"/>
+      <c r="N5" s="3"/>
+      <c r="O5" s="3"/>
+      <c r="P5" s="3"/>
+      <c r="Q5" s="3"/>
+      <c r="R5" s="3"/>
+      <c r="S5" s="3"/>
     </row>
     <row r="6" spans="1:19">
-      <c r="A6" s="1">
+      <c r="A6" s="3">
         <v>17</v>
       </c>
-      <c r="B6" s="1">
+      <c r="B6" s="3">
         <v>24</v>
       </c>
-      <c r="C6" s="1">
+      <c r="C6" s="3">
         <v>32</v>
       </c>
-      <c r="D6" s="1">
+      <c r="D6" s="3">
         <v>39</v>
       </c>
-      <c r="E6" s="1">
+      <c r="E6" s="3">
         <v>47</v>
       </c>
-      <c r="F6" s="1">
+      <c r="F6" s="3">
         <v>55</v>
       </c>
-      <c r="G6" s="1">
+      <c r="G6" s="3">
         <v>64</v>
       </c>
-      <c r="H6" s="1">
+      <c r="H6" s="3">
         <v>72</v>
       </c>
-      <c r="I6" s="1">
+      <c r="I6" s="3">
         <v>81</v>
       </c>
-      <c r="J6" s="1">
+      <c r="J6" s="3">
         <v>90</v>
       </c>
-      <c r="K6" s="1">
+      <c r="K6" s="3">
         <v>100</v>
       </c>
-      <c r="L6" s="1"/>
-      <c r="M6" s="1"/>
-      <c r="N6" s="1"/>
-      <c r="O6" s="1"/>
-      <c r="P6" s="1"/>
-      <c r="Q6" s="1"/>
-      <c r="R6" s="1"/>
-      <c r="S6" s="1"/>
+      <c r="L6" s="3"/>
+      <c r="M6" s="3"/>
+      <c r="N6" s="3"/>
+      <c r="O6" s="3"/>
+      <c r="P6" s="3"/>
+      <c r="Q6" s="3"/>
+      <c r="R6" s="3"/>
+      <c r="S6" s="3"/>
     </row>
     <row r="7" spans="1:19">
-      <c r="A7" s="1">
+      <c r="A7" s="3">
         <v>18</v>
       </c>
-      <c r="B7" s="1">
+      <c r="B7" s="3">
         <v>20</v>
       </c>
-      <c r="C7" s="1">
+      <c r="C7" s="3">
         <v>27</v>
       </c>
-      <c r="D7" s="1">
+      <c r="D7" s="3">
         <v>34</v>
       </c>
-      <c r="E7" s="1">
+      <c r="E7" s="3">
         <v>41</v>
       </c>
-      <c r="F7" s="1">
+      <c r="F7" s="3">
         <v>49</v>
       </c>
-      <c r="G7" s="1">
+      <c r="G7" s="3">
         <v>56</v>
       </c>
-      <c r="H7" s="1">
+      <c r="H7" s="3">
         <v>65</v>
       </c>
-      <c r="I7" s="1">
+      <c r="I7" s="3">
         <v>73</v>
       </c>
-      <c r="J7" s="1">
+      <c r="J7" s="3">
         <v>82</v>
       </c>
-      <c r="K7" s="1">
+      <c r="K7" s="3">
         <v>91</v>
       </c>
-      <c r="L7" s="1">
+      <c r="L7" s="3">
         <v>100</v>
       </c>
-      <c r="M7" s="1"/>
-      <c r="N7" s="1"/>
-      <c r="O7" s="1"/>
-      <c r="P7" s="1"/>
-      <c r="Q7" s="1"/>
-      <c r="R7" s="1"/>
-      <c r="S7" s="1"/>
+      <c r="M7" s="3"/>
+      <c r="N7" s="3"/>
+      <c r="O7" s="3"/>
+      <c r="P7" s="3"/>
+      <c r="Q7" s="3"/>
+      <c r="R7" s="3"/>
+      <c r="S7" s="3"/>
     </row>
     <row r="8" spans="1:19">
-      <c r="A8" s="1">
+      <c r="A8" s="3">
         <v>19</v>
       </c>
-      <c r="B8" s="1">
+      <c r="B8" s="3">
         <v>15</v>
       </c>
-      <c r="C8" s="1">
+      <c r="C8" s="3">
         <v>22</v>
       </c>
-      <c r="D8" s="1">
+      <c r="D8" s="3">
         <v>29</v>
       </c>
-      <c r="E8" s="1">
+      <c r="E8" s="3">
         <v>36</v>
       </c>
-      <c r="F8" s="1">
+      <c r="F8" s="3">
         <v>43</v>
       </c>
-      <c r="G8" s="1">
+      <c r="G8" s="3">
         <v>50</v>
       </c>
-      <c r="H8" s="1">
+      <c r="H8" s="3">
         <v>58</v>
       </c>
-      <c r="I8" s="1">
+      <c r="I8" s="3">
         <v>66</v>
       </c>
-      <c r="J8" s="1">
+      <c r="J8" s="3">
         <v>74</v>
       </c>
-      <c r="K8" s="1">
+      <c r="K8" s="3">
         <v>82</v>
       </c>
-      <c r="L8" s="1">
+      <c r="L8" s="3">
         <v>91</v>
       </c>
-      <c r="M8" s="1">
+      <c r="M8" s="3">
         <v>100</v>
       </c>
-      <c r="N8" s="1"/>
-      <c r="O8" s="1"/>
-      <c r="P8" s="1"/>
-      <c r="Q8" s="1"/>
-      <c r="R8" s="1"/>
-      <c r="S8" s="1"/>
+      <c r="N8" s="3"/>
+      <c r="O8" s="3"/>
+      <c r="P8" s="3"/>
+      <c r="Q8" s="3"/>
+      <c r="R8" s="3"/>
+      <c r="S8" s="3"/>
     </row>
     <row r="9" spans="1:19">
-      <c r="A9" s="1">
+      <c r="A9" s="3">
         <v>20</v>
       </c>
-      <c r="B9" s="1"/>
-      <c r="C9" s="1">
+      <c r="B9" s="3"/>
+      <c r="C9" s="3">
         <v>18</v>
       </c>
-      <c r="D9" s="1">
+      <c r="D9" s="3">
         <v>24</v>
       </c>
-      <c r="E9" s="1">
+      <c r="E9" s="3">
         <v>30</v>
       </c>
-      <c r="F9" s="1">
+      <c r="F9" s="3">
         <v>37</v>
       </c>
-      <c r="G9" s="1">
+      <c r="G9" s="3">
         <v>44</v>
       </c>
-      <c r="H9" s="1">
+      <c r="H9" s="3">
         <v>52</v>
       </c>
-      <c r="I9" s="1">
+      <c r="I9" s="3">
         <v>59</v>
       </c>
-      <c r="J9" s="1">
+      <c r="J9" s="3">
         <v>66</v>
       </c>
-      <c r="K9" s="1">
+      <c r="K9" s="3">
         <v>74</v>
       </c>
-      <c r="L9" s="1">
+      <c r="L9" s="3">
         <v>83</v>
       </c>
-      <c r="M9" s="1">
+      <c r="M9" s="3">
         <v>91</v>
       </c>
-      <c r="N9" s="1">
+      <c r="N9" s="3">
         <v>100</v>
       </c>
-      <c r="O9" s="1"/>
-      <c r="P9" s="1"/>
-      <c r="Q9" s="1"/>
-      <c r="R9" s="1"/>
-      <c r="S9" s="1"/>
+      <c r="O9" s="3"/>
+      <c r="P9" s="3"/>
+      <c r="Q9" s="3"/>
+      <c r="R9" s="3"/>
+      <c r="S9" s="3"/>
     </row>
     <row r="10" spans="1:19">
-      <c r="A10" s="1">
+      <c r="A10" s="3">
         <v>21</v>
       </c>
-      <c r="B10" s="1"/>
-      <c r="C10" s="1">
+      <c r="B10" s="3"/>
+      <c r="C10" s="3">
         <v>14</v>
       </c>
-      <c r="D10" s="1">
+      <c r="D10" s="3">
         <v>20</v>
       </c>
-      <c r="E10" s="1">
+      <c r="E10" s="3">
         <v>26</v>
       </c>
-      <c r="F10" s="1">
+      <c r="F10" s="3">
         <v>32</v>
       </c>
-      <c r="G10" s="1">
+      <c r="G10" s="3">
         <v>39</v>
       </c>
-      <c r="H10" s="1">
+      <c r="H10" s="3">
         <v>46</v>
       </c>
-      <c r="I10" s="1">
+      <c r="I10" s="3">
         <v>53</v>
       </c>
-      <c r="J10" s="1">
+      <c r="J10" s="3">
         <v>60</v>
       </c>
-      <c r="K10" s="1">
+      <c r="K10" s="3">
         <v>67</v>
       </c>
-      <c r="L10" s="1">
+      <c r="L10" s="3">
         <v>75</v>
       </c>
-      <c r="M10" s="1">
+      <c r="M10" s="3">
         <v>83</v>
       </c>
-      <c r="N10" s="1">
+      <c r="N10" s="3">
         <v>91</v>
       </c>
-      <c r="O10" s="1">
+      <c r="O10" s="3">
         <v>100</v>
       </c>
-      <c r="P10" s="1"/>
-      <c r="Q10" s="1"/>
-      <c r="R10" s="1"/>
-      <c r="S10" s="1"/>
+      <c r="P10" s="3"/>
+      <c r="Q10" s="3"/>
+      <c r="R10" s="3"/>
+      <c r="S10" s="3"/>
     </row>
     <row r="11" spans="1:19">
-      <c r="A11" s="1">
+      <c r="A11" s="3">
         <v>22</v>
       </c>
-      <c r="B11" s="1"/>
-      <c r="C11" s="1"/>
-      <c r="D11" s="1">
+      <c r="B11" s="3"/>
+      <c r="C11" s="3"/>
+      <c r="D11" s="3">
         <v>16</v>
       </c>
-      <c r="E11" s="1">
+      <c r="E11" s="3">
         <v>22</v>
       </c>
-      <c r="F11" s="1">
+      <c r="F11" s="3">
         <v>28</v>
       </c>
-      <c r="G11" s="1">
+      <c r="G11" s="3">
         <v>34</v>
       </c>
-      <c r="H11" s="1">
+      <c r="H11" s="3">
         <v>40</v>
       </c>
-      <c r="I11" s="1">
+      <c r="I11" s="3">
         <v>47</v>
       </c>
-      <c r="J11" s="1">
+      <c r="J11" s="3">
         <v>54</v>
       </c>
-      <c r="K11" s="1">
+      <c r="K11" s="3">
         <v>61</v>
       </c>
-      <c r="L11" s="1">
+      <c r="L11" s="3">
         <v>68</v>
       </c>
-      <c r="M11" s="1">
+      <c r="M11" s="3">
         <v>76</v>
       </c>
-      <c r="N11" s="1">
+      <c r="N11" s="3">
         <v>84</v>
       </c>
-      <c r="O11" s="1">
+      <c r="O11" s="3">
         <v>92</v>
       </c>
-      <c r="P11" s="1">
+      <c r="P11" s="3">
         <v>100</v>
       </c>
-      <c r="Q11" s="1"/>
-      <c r="R11" s="1"/>
-      <c r="S11" s="1"/>
+      <c r="Q11" s="3"/>
+      <c r="R11" s="3"/>
+      <c r="S11" s="3"/>
     </row>
     <row r="12" spans="1:19">
-      <c r="A12" s="1">
+      <c r="A12" s="3">
         <v>23</v>
       </c>
-      <c r="B12" s="1"/>
-      <c r="C12" s="1"/>
-      <c r="D12" s="1">
+      <c r="B12" s="3"/>
+      <c r="C12" s="3"/>
+      <c r="D12" s="3">
         <v>13</v>
       </c>
-      <c r="E12" s="1">
+      <c r="E12" s="3">
         <v>18</v>
       </c>
-      <c r="F12" s="1">
+      <c r="F12" s="3">
         <v>24</v>
       </c>
-      <c r="G12" s="1">
+      <c r="G12" s="3">
         <v>30</v>
       </c>
-      <c r="H12" s="1">
+      <c r="H12" s="3">
         <v>36</v>
       </c>
-      <c r="I12" s="1">
+      <c r="I12" s="3">
         <v>42</v>
       </c>
-      <c r="J12" s="1">
+      <c r="J12" s="3">
         <v>48</v>
       </c>
-      <c r="K12" s="1">
+      <c r="K12" s="3">
         <v>55</v>
       </c>
-      <c r="L12" s="1">
+      <c r="L12" s="3">
         <v>62</v>
       </c>
-      <c r="M12" s="1">
+      <c r="M12" s="3">
         <v>69</v>
       </c>
-      <c r="N12" s="1">
+      <c r="N12" s="3">
         <v>76</v>
       </c>
-      <c r="O12" s="1">
+      <c r="O12" s="3">
         <v>84</v>
       </c>
-      <c r="P12" s="1">
+      <c r="P12" s="3">
         <v>92</v>
       </c>
-      <c r="Q12" s="1">
+      <c r="Q12" s="3">
         <v>100</v>
       </c>
-      <c r="R12" s="1"/>
-      <c r="S12" s="1"/>
+      <c r="R12" s="3"/>
+      <c r="S12" s="3"/>
     </row>
     <row r="13" spans="1:19">
-      <c r="A13" s="1">
+      <c r="A13" s="3">
         <v>24</v>
       </c>
-      <c r="B13" s="1"/>
-      <c r="C13" s="1"/>
-      <c r="D13" s="1"/>
-      <c r="E13" s="1">
+      <c r="B13" s="3"/>
+      <c r="C13" s="3"/>
+      <c r="D13" s="3"/>
+      <c r="E13" s="3">
         <v>15</v>
       </c>
-      <c r="F13" s="1">
+      <c r="F13" s="3">
         <v>20</v>
       </c>
-      <c r="G13" s="1">
+      <c r="G13" s="3">
         <v>26</v>
       </c>
-      <c r="H13" s="1">
+      <c r="H13" s="3">
         <v>31</v>
       </c>
-      <c r="I13" s="1">
+      <c r="I13" s="3">
         <v>37</v>
       </c>
-      <c r="J13" s="1">
+      <c r="J13" s="3">
         <v>43</v>
       </c>
-      <c r="K13" s="1">
+      <c r="K13" s="3">
         <v>49</v>
       </c>
-      <c r="L13" s="1">
+      <c r="L13" s="3">
         <v>56</v>
       </c>
-      <c r="M13" s="1">
+      <c r="M13" s="3">
         <v>63</v>
       </c>
-      <c r="N13" s="1">
+      <c r="N13" s="3">
         <v>70</v>
       </c>
-      <c r="O13" s="1">
+      <c r="O13" s="3">
         <v>77</v>
       </c>
-      <c r="P13" s="1">
+      <c r="P13" s="3">
         <v>84</v>
       </c>
-      <c r="Q13" s="1">
+      <c r="Q13" s="3">
         <v>92</v>
       </c>
-      <c r="R13" s="1">
+      <c r="R13" s="3">
         <v>100</v>
       </c>
-      <c r="S13" s="1"/>
+      <c r="S13" s="3"/>
     </row>
     <row r="14" spans="1:19">
-      <c r="A14" s="1">
+      <c r="A14" s="3">
         <v>25</v>
       </c>
-      <c r="B14" s="1"/>
-      <c r="C14" s="1"/>
-      <c r="D14" s="1"/>
-      <c r="E14" s="1"/>
-      <c r="F14" s="1">
+      <c r="B14" s="3"/>
+      <c r="C14" s="3"/>
+      <c r="D14" s="3"/>
+      <c r="E14" s="3"/>
+      <c r="F14" s="3">
         <v>17</v>
       </c>
-      <c r="G14" s="1">
+      <c r="G14" s="3">
         <v>22</v>
       </c>
-      <c r="H14" s="1">
+      <c r="H14" s="3">
         <v>27</v>
       </c>
-      <c r="I14" s="1">
+      <c r="I14" s="3">
         <v>33</v>
       </c>
-      <c r="J14" s="1">
+      <c r="J14" s="3">
         <v>38</v>
       </c>
-      <c r="K14" s="1">
+      <c r="K14" s="3">
         <v>44</v>
       </c>
-      <c r="L14" s="1">
+      <c r="L14" s="3">
         <v>50</v>
       </c>
-      <c r="M14" s="1">
+      <c r="M14" s="3">
         <v>57</v>
       </c>
-      <c r="N14" s="1">
+      <c r="N14" s="3">
         <v>63</v>
       </c>
-      <c r="O14" s="1">
+      <c r="O14" s="3">
         <v>70</v>
       </c>
-      <c r="P14" s="1">
+      <c r="P14" s="3">
         <v>77</v>
       </c>
-      <c r="Q14" s="1">
+      <c r="Q14" s="3">
         <v>84</v>
       </c>
-      <c r="R14" s="1">
+      <c r="R14" s="3">
         <v>92</v>
       </c>
-      <c r="S14" s="1">
+      <c r="S14" s="3">
         <v>100</v>
       </c>
     </row>
     <row r="15" spans="1:19">
-      <c r="A15" s="1">
+      <c r="A15" s="3">
         <v>26</v>
       </c>
-      <c r="B15" s="1"/>
-      <c r="C15" s="1"/>
-      <c r="D15" s="1"/>
-      <c r="E15" s="1"/>
-      <c r="F15" s="1">
+      <c r="B15" s="3"/>
+      <c r="C15" s="3"/>
+      <c r="D15" s="3"/>
+      <c r="E15" s="3"/>
+      <c r="F15" s="3">
         <v>14</v>
       </c>
-      <c r="G15" s="1">
+      <c r="G15" s="3">
         <v>19</v>
       </c>
-      <c r="H15" s="1">
+      <c r="H15" s="3">
         <v>24</v>
       </c>
-      <c r="I15" s="1">
+      <c r="I15" s="3">
         <v>29</v>
       </c>
-      <c r="J15" s="1">
+      <c r="J15" s="3">
         <v>34</v>
       </c>
-      <c r="K15" s="1">
+      <c r="K15" s="3">
         <v>40</v>
       </c>
-      <c r="L15" s="1">
+      <c r="L15" s="3">
         <v>46</v>
       </c>
-      <c r="M15" s="1">
+      <c r="M15" s="3">
         <v>52</v>
       </c>
-      <c r="N15" s="1">
+      <c r="N15" s="3">
         <v>57</v>
       </c>
-      <c r="O15" s="1">
+      <c r="O15" s="3">
         <v>64</v>
       </c>
-      <c r="P15" s="1">
+      <c r="P15" s="3">
         <v>71</v>
       </c>
-      <c r="Q15" s="1">
+      <c r="Q15" s="3">
         <v>77</v>
       </c>
-      <c r="R15" s="1">
+      <c r="R15" s="3">
         <v>85</v>
       </c>
-      <c r="S15" s="1">
+      <c r="S15" s="3">
         <v>92</v>
       </c>
     </row>
     <row r="16" spans="1:19">
-      <c r="A16" s="1">
+      <c r="A16" s="3">
         <v>27</v>
       </c>
-      <c r="B16" s="1"/>
-      <c r="C16" s="1"/>
-      <c r="D16" s="1"/>
-      <c r="E16" s="1"/>
-      <c r="F16" s="1"/>
-      <c r="G16" s="1">
+      <c r="B16" s="3"/>
+      <c r="C16" s="3"/>
+      <c r="D16" s="3"/>
+      <c r="E16" s="3"/>
+      <c r="F16" s="3"/>
+      <c r="G16" s="3">
         <v>16</v>
       </c>
-      <c r="H16" s="1">
+      <c r="H16" s="3">
         <v>21</v>
       </c>
-      <c r="I16" s="1">
+      <c r="I16" s="3">
         <v>25</v>
       </c>
-      <c r="J16" s="1">
+      <c r="J16" s="3">
         <v>30</v>
       </c>
-      <c r="K16" s="1">
+      <c r="K16" s="3">
         <v>36</v>
       </c>
-      <c r="L16" s="1">
+      <c r="L16" s="3">
         <v>41</v>
       </c>
-      <c r="M16" s="1">
+      <c r="M16" s="3">
         <v>47</v>
       </c>
-      <c r="N16" s="1">
+      <c r="N16" s="3">
         <v>52</v>
       </c>
-      <c r="O16" s="1">
+      <c r="O16" s="3">
         <v>58</v>
       </c>
-      <c r="P16" s="1">
+      <c r="P16" s="3">
         <v>65</v>
       </c>
-      <c r="Q16" s="1">
+      <c r="Q16" s="3">
         <v>71</v>
       </c>
-      <c r="R16" s="1">
+      <c r="R16" s="3">
         <v>78</v>
       </c>
-      <c r="S16" s="1">
+      <c r="S16" s="3">
         <v>85</v>
       </c>
     </row>

</xml_diff>